<commit_message>
added NonNative and Bot
Only flagged one as bot, quite a few possible non-native participants. I put "?" to some, please do check.
</commit_message>
<xml_diff>
--- a/output/papers/Round 2/CISP_data_participant-comments.xlsx
+++ b/output/papers/Round 2/CISP_data_participant-comments.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gekagrob/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{1FA9CDA1-F8DF-4847-9653-BC2CD808C17E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AFC2179-6B84-9346-8565-46CA72ADE197}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="30240" windowHeight="18900" xr2:uid="{73614858-1B18-2D48-8B46-604ABCED0ED9}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17920" xr2:uid="{73614858-1B18-2D48-8B46-604ABCED0ED9}"/>
   </bookViews>
   <sheets>
     <sheet name="CISP_data_participant-comments" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1088" uniqueCount="536">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1111" uniqueCount="542">
   <si>
     <t>Experiment</t>
   </si>
@@ -1633,13 +1633,31 @@
   </si>
   <si>
     <t>No, I did not notice anything strange in her to be honest</t>
+  </si>
+  <si>
+    <t>Talker.SpeechDescription_NonNative</t>
+  </si>
+  <si>
+    <t>Talker.SpeechDescription_Bot</t>
+  </si>
+  <si>
+    <t>?</t>
+  </si>
+  <si>
+    <t>? (same comment, same punctuation)</t>
+  </si>
+  <si>
+    <t>? (could be a typo)</t>
+  </si>
+  <si>
+    <t>? (common mistake among natives too, not sure)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="22" x14ac:knownFonts="1">
+  <fonts count="21" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1779,12 +1797,6 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Helvetica Neue"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="12"/>
@@ -2140,7 +2152,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -2149,13 +2161,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2533,7 +2538,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A55A15C-6534-3841-BFC9-6C6D5C268A75}">
-  <dimension ref="A1:K834"/>
+  <dimension ref="A1:M834"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="22.33203125" customWidth="1"/>
@@ -2547,9 +2552,11 @@
     <col min="9" max="9" width="48.83203125" customWidth="1"/>
     <col min="10" max="10" width="34" customWidth="1"/>
     <col min="11" max="11" width="35" customWidth="1"/>
+    <col min="12" max="12" width="44.83203125" customWidth="1"/>
+    <col min="13" max="13" width="32" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2583,8 +2590,14 @@
       <c r="K1" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" ht="68" x14ac:dyDescent="0.2">
+      <c r="L1" t="s">
+        <v>536</v>
+      </c>
+      <c r="M1" t="s">
+        <v>537</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" ht="68" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -2599,7 +2612,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -2614,7 +2627,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="34" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:13" ht="34" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>11</v>
       </c>
@@ -2626,7 +2639,7 @@
       </c>
       <c r="D4" s="1"/>
     </row>
-    <row r="5" spans="1:11" ht="51" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:13" ht="51" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>11</v>
       </c>
@@ -2644,7 +2657,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>11</v>
       </c>
@@ -2659,7 +2672,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>11</v>
       </c>
@@ -2669,7 +2682,7 @@
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
     </row>
-    <row r="8" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -2681,7 +2694,7 @@
       </c>
       <c r="D8" s="1"/>
     </row>
-    <row r="9" spans="1:11" ht="51" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:13" ht="51" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>11</v>
       </c>
@@ -2696,7 +2709,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>11</v>
       </c>
@@ -2708,7 +2721,7 @@
       </c>
       <c r="D10" s="1"/>
     </row>
-    <row r="11" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>11</v>
       </c>
@@ -2723,7 +2736,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="51" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:13" ht="51" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>11</v>
       </c>
@@ -2738,7 +2751,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>11</v>
       </c>
@@ -2750,7 +2763,7 @@
       </c>
       <c r="D13" s="1"/>
     </row>
-    <row r="14" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>11</v>
       </c>
@@ -2762,7 +2775,7 @@
       </c>
       <c r="D14" s="1"/>
     </row>
-    <row r="15" spans="1:11" ht="68" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:13" ht="68" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>11</v>
       </c>
@@ -2783,7 +2796,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:11" ht="34" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:13" ht="34" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>11</v>
       </c>
@@ -2797,7 +2810,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="17" spans="1:10" ht="34" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>11</v>
       </c>
@@ -2811,8 +2824,11 @@
       <c r="E17" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="18" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+      <c r="L17" t="s">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>11</v>
       </c>
@@ -2824,7 +2840,7 @@
       </c>
       <c r="D18" s="1"/>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>11</v>
       </c>
@@ -2834,7 +2850,7 @@
       <c r="C19" s="1"/>
       <c r="D19" s="1"/>
     </row>
-    <row r="20" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>11</v>
       </c>
@@ -2849,7 +2865,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="21" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>11</v>
       </c>
@@ -2864,7 +2880,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="22" spans="1:10" ht="34" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>11</v>
       </c>
@@ -2882,7 +2898,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="23" spans="1:10" ht="51" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:12" ht="51" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>11</v>
       </c>
@@ -2894,7 +2910,7 @@
       </c>
       <c r="D23" s="1"/>
     </row>
-    <row r="24" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>11</v>
       </c>
@@ -2906,7 +2922,7 @@
       </c>
       <c r="D24" s="1"/>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>11</v>
       </c>
@@ -2916,7 +2932,7 @@
       <c r="C25" s="1"/>
       <c r="D25" s="1"/>
     </row>
-    <row r="26" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>11</v>
       </c>
@@ -2928,7 +2944,7 @@
       </c>
       <c r="D26" s="1"/>
     </row>
-    <row r="27" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>11</v>
       </c>
@@ -2943,7 +2959,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="28" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>11</v>
       </c>
@@ -2958,7 +2974,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="29" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>11</v>
       </c>
@@ -2970,7 +2986,7 @@
       </c>
       <c r="D29" s="1"/>
     </row>
-    <row r="30" spans="1:10" ht="34" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>11</v>
       </c>
@@ -2987,8 +3003,11 @@
       <c r="H30" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="31" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+      <c r="L30" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>11</v>
       </c>
@@ -3000,7 +3019,7 @@
       </c>
       <c r="D31" s="1"/>
     </row>
-    <row r="32" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>11</v>
       </c>
@@ -3015,7 +3034,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="33" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>11</v>
       </c>
@@ -3030,7 +3049,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="34" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>11</v>
       </c>
@@ -3042,7 +3061,7 @@
       </c>
       <c r="D34" s="1"/>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>11</v>
       </c>
@@ -3052,7 +3071,7 @@
       <c r="C35" s="1"/>
       <c r="D35" s="1"/>
     </row>
-    <row r="36" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>11</v>
       </c>
@@ -3064,7 +3083,7 @@
       </c>
       <c r="D36" s="1"/>
     </row>
-    <row r="37" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>11</v>
       </c>
@@ -3076,7 +3095,7 @@
       </c>
       <c r="D37" s="1"/>
     </row>
-    <row r="38" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>11</v>
       </c>
@@ -3088,7 +3107,7 @@
       </c>
       <c r="D38" s="1"/>
     </row>
-    <row r="39" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>11</v>
       </c>
@@ -3100,7 +3119,7 @@
       </c>
       <c r="D39" s="1"/>
     </row>
-    <row r="40" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>11</v>
       </c>
@@ -3114,7 +3133,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="41" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>11</v>
       </c>
@@ -3127,8 +3146,11 @@
       <c r="D41" s="1" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L41" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>11</v>
       </c>
@@ -3138,7 +3160,7 @@
       <c r="C42" s="1"/>
       <c r="D42" s="1"/>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>11</v>
       </c>
@@ -3148,7 +3170,7 @@
       <c r="C43" s="1"/>
       <c r="D43" s="1"/>
     </row>
-    <row r="44" spans="1:10" ht="34" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>11</v>
       </c>
@@ -3166,7 +3188,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="45" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>11</v>
       </c>
@@ -3178,7 +3200,7 @@
       </c>
       <c r="D45" s="1"/>
     </row>
-    <row r="46" spans="1:10" ht="34" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>11</v>
       </c>
@@ -3193,7 +3215,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>11</v>
       </c>
@@ -3203,7 +3225,7 @@
       <c r="C47" s="1"/>
       <c r="D47" s="1"/>
     </row>
-    <row r="48" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>11</v>
       </c>
@@ -3893,7 +3915,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="97" spans="1:6" ht="34" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
         <v>118</v>
       </c>
@@ -3908,7 +3930,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="98" spans="1:6" ht="34" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
         <v>118</v>
       </c>
@@ -3922,8 +3944,11 @@
       <c r="F98" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="99" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+      <c r="L98" t="s">
+        <v>541</v>
+      </c>
+    </row>
+    <row r="99" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
         <v>118</v>
       </c>
@@ -3938,7 +3963,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="100" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
         <v>118</v>
       </c>
@@ -3953,7 +3978,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="101" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
         <v>118</v>
       </c>
@@ -3968,7 +3993,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="102" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
         <v>118</v>
       </c>
@@ -3980,7 +4005,7 @@
       </c>
       <c r="D102" s="1"/>
     </row>
-    <row r="103" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
         <v>118</v>
       </c>
@@ -3992,7 +4017,7 @@
       </c>
       <c r="D103" s="1"/>
     </row>
-    <row r="104" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
         <v>118</v>
       </c>
@@ -4004,7 +4029,7 @@
       </c>
       <c r="D104" s="1"/>
     </row>
-    <row r="105" spans="1:6" ht="68" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:12" ht="68" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
         <v>118</v>
       </c>
@@ -4021,7 +4046,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="106" spans="1:6" ht="34" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
         <v>118</v>
       </c>
@@ -4036,7 +4061,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
         <v>118</v>
       </c>
@@ -4046,7 +4071,7 @@
       <c r="C107" s="1"/>
       <c r="D107" s="1"/>
     </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
         <v>118</v>
       </c>
@@ -4056,7 +4081,7 @@
       <c r="C108" s="1"/>
       <c r="D108" s="1"/>
     </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
         <v>118</v>
       </c>
@@ -4066,7 +4091,7 @@
       <c r="C109" s="1"/>
       <c r="D109" s="1"/>
     </row>
-    <row r="110" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:12" ht="51" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
         <v>118</v>
       </c>
@@ -4084,7 +4109,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="111" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
         <v>118</v>
       </c>
@@ -4099,7 +4124,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="112" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
         <v>118</v>
       </c>
@@ -5034,7 +5059,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="177" spans="1:11" ht="119" x14ac:dyDescent="0.2">
+    <row r="177" spans="1:13" ht="119" x14ac:dyDescent="0.2">
       <c r="A177" t="s">
         <v>219</v>
       </c>
@@ -5052,7 +5077,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="178" spans="1:11" ht="34" x14ac:dyDescent="0.2">
+    <row r="178" spans="1:13" ht="34" x14ac:dyDescent="0.2">
       <c r="A178" t="s">
         <v>219</v>
       </c>
@@ -5070,33 +5095,26 @@
         <v>14</v>
       </c>
     </row>
-    <row r="179" spans="1:11" ht="17" x14ac:dyDescent="0.2">
-      <c r="A179" s="5" t="s">
+    <row r="179" spans="1:13" ht="17" x14ac:dyDescent="0.2">
+      <c r="A179" t="s">
         <v>326</v>
       </c>
-      <c r="B179" s="5" t="s">
+      <c r="B179" t="s">
         <v>327</v>
       </c>
-      <c r="C179" s="6" t="s">
+      <c r="C179" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="D179" s="6"/>
-      <c r="E179" s="5"/>
-      <c r="F179" s="5"/>
-      <c r="G179" s="5"/>
-      <c r="H179" s="5"/>
-      <c r="I179" s="5"/>
-      <c r="J179" s="5"/>
-      <c r="K179" s="5"/>
-    </row>
-    <row r="180" spans="1:11" ht="29" x14ac:dyDescent="0.2">
+      <c r="D179" s="1"/>
+    </row>
+    <row r="180" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A180" t="s">
         <v>326</v>
       </c>
       <c r="B180" t="s">
         <v>328</v>
       </c>
-      <c r="C180" s="2" t="s">
+      <c r="C180" s="3" t="s">
         <v>391</v>
       </c>
       <c r="D180" s="1"/>
@@ -5104,40 +5122,40 @@
         <v>14</v>
       </c>
     </row>
-    <row r="181" spans="1:11" ht="43" x14ac:dyDescent="0.2">
+    <row r="181" spans="1:13" ht="51" x14ac:dyDescent="0.2">
       <c r="A181" t="s">
         <v>326</v>
       </c>
       <c r="B181" t="s">
         <v>329</v>
       </c>
-      <c r="C181" s="2" t="s">
+      <c r="C181" s="3" t="s">
         <v>392</v>
       </c>
       <c r="D181" s="1"/>
     </row>
-    <row r="182" spans="1:11" ht="29" x14ac:dyDescent="0.2">
+    <row r="182" spans="1:13" ht="34" x14ac:dyDescent="0.2">
       <c r="A182" t="s">
         <v>326</v>
       </c>
       <c r="B182" t="s">
         <v>330</v>
       </c>
-      <c r="C182" s="2" t="s">
+      <c r="C182" s="3" t="s">
         <v>393</v>
       </c>
       <c r="D182" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="183" spans="1:11" ht="34" x14ac:dyDescent="0.2">
+    <row r="183" spans="1:13" ht="34" x14ac:dyDescent="0.2">
       <c r="A183" t="s">
         <v>326</v>
       </c>
       <c r="B183" t="s">
         <v>331</v>
       </c>
-      <c r="C183" s="4" t="s">
+      <c r="C183" s="3" t="s">
         <v>394</v>
       </c>
       <c r="D183" s="1"/>
@@ -5145,38 +5163,41 @@
         <v>14</v>
       </c>
     </row>
-    <row r="184" spans="1:11" ht="34" x14ac:dyDescent="0.2">
+    <row r="184" spans="1:13" ht="34" x14ac:dyDescent="0.2">
       <c r="A184" t="s">
         <v>326</v>
       </c>
       <c r="B184" t="s">
         <v>332</v>
       </c>
-      <c r="C184" s="4" t="s">
+      <c r="C184" s="3" t="s">
         <v>395</v>
       </c>
       <c r="D184" s="1"/>
-    </row>
-    <row r="185" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+      <c r="M184" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="185" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A185" t="s">
         <v>326</v>
       </c>
       <c r="B185" t="s">
         <v>333</v>
       </c>
-      <c r="C185" s="3" t="s">
+      <c r="C185" s="2" t="s">
         <v>29</v>
       </c>
       <c r="D185" s="1"/>
     </row>
-    <row r="186" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+    <row r="186" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A186" t="s">
         <v>326</v>
       </c>
       <c r="B186" t="s">
         <v>334</v>
       </c>
-      <c r="C186" s="4" t="s">
+      <c r="C186" s="3" t="s">
         <v>396</v>
       </c>
       <c r="D186" s="1"/>
@@ -5184,77 +5205,83 @@
         <v>14</v>
       </c>
     </row>
-    <row r="187" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+    <row r="187" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A187" t="s">
         <v>326</v>
       </c>
       <c r="B187" t="s">
         <v>335</v>
       </c>
-      <c r="C187" s="4" t="s">
+      <c r="C187" s="3" t="s">
         <v>397</v>
       </c>
       <c r="D187" s="1" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="188" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L187" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="188" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A188" t="s">
         <v>326</v>
       </c>
       <c r="B188" t="s">
         <v>336</v>
       </c>
-      <c r="C188" s="3"/>
+      <c r="C188" s="2"/>
       <c r="D188" s="1"/>
     </row>
-    <row r="189" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+    <row r="189" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A189" t="s">
         <v>326</v>
       </c>
       <c r="B189" t="s">
         <v>337</v>
       </c>
-      <c r="C189" s="4" t="s">
+      <c r="C189" s="3" t="s">
         <v>398</v>
       </c>
       <c r="D189" s="1"/>
       <c r="K189" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="190" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+      <c r="L189" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="190" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A190" t="s">
         <v>326</v>
       </c>
       <c r="B190" t="s">
         <v>338</v>
       </c>
-      <c r="C190" s="3" t="s">
+      <c r="C190" s="2" t="s">
         <v>29</v>
       </c>
       <c r="D190" s="1"/>
     </row>
-    <row r="191" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+    <row r="191" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A191" t="s">
         <v>326</v>
       </c>
       <c r="B191" t="s">
         <v>339</v>
       </c>
-      <c r="C191" s="3" t="s">
+      <c r="C191" s="2" t="s">
         <v>35</v>
       </c>
       <c r="D191" s="1"/>
     </row>
-    <row r="192" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+    <row r="192" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A192" t="s">
         <v>326</v>
       </c>
       <c r="B192" t="s">
         <v>340</v>
       </c>
-      <c r="C192" s="4" t="s">
+      <c r="C192" s="3" t="s">
         <v>399</v>
       </c>
       <c r="D192" s="1"/>
@@ -5266,7 +5293,7 @@
       <c r="B193" t="s">
         <v>341</v>
       </c>
-      <c r="C193" s="3" t="s">
+      <c r="C193" s="2" t="s">
         <v>400</v>
       </c>
       <c r="D193" s="1"/>
@@ -5278,7 +5305,7 @@
       <c r="B194" t="s">
         <v>342</v>
       </c>
-      <c r="C194" s="4" t="s">
+      <c r="C194" s="3" t="s">
         <v>401</v>
       </c>
       <c r="D194" s="1"/>
@@ -5290,7 +5317,7 @@
       <c r="B195" t="s">
         <v>343</v>
       </c>
-      <c r="C195" s="4" t="s">
+      <c r="C195" s="3" t="s">
         <v>402</v>
       </c>
       <c r="D195" s="1"/>
@@ -5302,7 +5329,7 @@
       <c r="B196" t="s">
         <v>344</v>
       </c>
-      <c r="C196" s="3" t="s">
+      <c r="C196" s="2" t="s">
         <v>35</v>
       </c>
       <c r="D196" s="1"/>
@@ -5314,7 +5341,7 @@
       <c r="B197" t="s">
         <v>345</v>
       </c>
-      <c r="C197" s="3" t="s">
+      <c r="C197" s="2" t="s">
         <v>403</v>
       </c>
       <c r="D197" s="1" t="s">
@@ -5331,7 +5358,7 @@
       <c r="B198" t="s">
         <v>346</v>
       </c>
-      <c r="C198" s="3" t="s">
+      <c r="C198" s="2" t="s">
         <v>35</v>
       </c>
       <c r="D198" s="1"/>
@@ -5343,7 +5370,7 @@
       <c r="B199" t="s">
         <v>347</v>
       </c>
-      <c r="C199" s="3" t="s">
+      <c r="C199" s="2" t="s">
         <v>404</v>
       </c>
       <c r="F199" t="s">
@@ -5357,7 +5384,7 @@
       <c r="B200" t="s">
         <v>348</v>
       </c>
-      <c r="C200" s="3" t="s">
+      <c r="C200" s="2" t="s">
         <v>35</v>
       </c>
     </row>
@@ -5368,7 +5395,7 @@
       <c r="B201" t="s">
         <v>349</v>
       </c>
-      <c r="C201" s="4" t="s">
+      <c r="C201" s="3" t="s">
         <v>405</v>
       </c>
       <c r="F201" t="s">
@@ -5382,7 +5409,7 @@
       <c r="B202" t="s">
         <v>350</v>
       </c>
-      <c r="C202" s="3" t="s">
+      <c r="C202" s="2" t="s">
         <v>400</v>
       </c>
     </row>
@@ -5393,7 +5420,7 @@
       <c r="B203" t="s">
         <v>351</v>
       </c>
-      <c r="C203" s="4" t="s">
+      <c r="C203" s="3" t="s">
         <v>406</v>
       </c>
       <c r="F203" t="s">
@@ -5407,7 +5434,7 @@
       <c r="B204" t="s">
         <v>352</v>
       </c>
-      <c r="C204" s="4" t="s">
+      <c r="C204" s="3" t="s">
         <v>407</v>
       </c>
       <c r="F204" t="s">
@@ -5421,7 +5448,7 @@
       <c r="B205" t="s">
         <v>353</v>
       </c>
-      <c r="C205" s="4" t="s">
+      <c r="C205" s="3" t="s">
         <v>408</v>
       </c>
       <c r="D205" t="s">
@@ -5435,7 +5462,7 @@
       <c r="B206" t="s">
         <v>354</v>
       </c>
-      <c r="C206" s="3" t="s">
+      <c r="C206" s="2" t="s">
         <v>35</v>
       </c>
     </row>
@@ -5446,7 +5473,7 @@
       <c r="B207" t="s">
         <v>355</v>
       </c>
-      <c r="C207" s="4" t="s">
+      <c r="C207" s="3" t="s">
         <v>409</v>
       </c>
       <c r="F207" t="s">
@@ -5460,7 +5487,7 @@
       <c r="B208" t="s">
         <v>356</v>
       </c>
-      <c r="C208" s="4" t="s">
+      <c r="C208" s="3" t="s">
         <v>410</v>
       </c>
       <c r="E208" t="s">
@@ -5474,7 +5501,7 @@
       <c r="B209" t="s">
         <v>357</v>
       </c>
-      <c r="C209" s="3" t="s">
+      <c r="C209" s="2" t="s">
         <v>411</v>
       </c>
     </row>
@@ -5485,7 +5512,7 @@
       <c r="B210" t="s">
         <v>358</v>
       </c>
-      <c r="C210" s="4" t="s">
+      <c r="C210" s="3" t="s">
         <v>412</v>
       </c>
     </row>
@@ -5496,7 +5523,7 @@
       <c r="B211" t="s">
         <v>359</v>
       </c>
-      <c r="C211" s="4" t="s">
+      <c r="C211" s="3" t="s">
         <v>413</v>
       </c>
       <c r="F211" t="s">
@@ -5510,7 +5537,7 @@
       <c r="B212" t="s">
         <v>360</v>
       </c>
-      <c r="C212" s="3" t="s">
+      <c r="C212" s="2" t="s">
         <v>414</v>
       </c>
     </row>
@@ -5521,7 +5548,7 @@
       <c r="B213" t="s">
         <v>361</v>
       </c>
-      <c r="C213" s="4" t="s">
+      <c r="C213" s="3" t="s">
         <v>415</v>
       </c>
       <c r="F213" t="s">
@@ -5535,7 +5562,7 @@
       <c r="B214" t="s">
         <v>362</v>
       </c>
-      <c r="C214" s="4" t="s">
+      <c r="C214" s="3" t="s">
         <v>416</v>
       </c>
     </row>
@@ -5546,7 +5573,7 @@
       <c r="B215" t="s">
         <v>363</v>
       </c>
-      <c r="C215" s="4" t="s">
+      <c r="C215" s="3" t="s">
         <v>411</v>
       </c>
     </row>
@@ -5557,7 +5584,7 @@
       <c r="B216" t="s">
         <v>364</v>
       </c>
-      <c r="C216" s="4" t="s">
+      <c r="C216" s="3" t="s">
         <v>417</v>
       </c>
     </row>
@@ -5568,7 +5595,7 @@
       <c r="B217" t="s">
         <v>365</v>
       </c>
-      <c r="C217" s="4" t="s">
+      <c r="C217" s="3" t="s">
         <v>418</v>
       </c>
     </row>
@@ -5579,7 +5606,7 @@
       <c r="B218" t="s">
         <v>366</v>
       </c>
-      <c r="C218" s="3" t="s">
+      <c r="C218" s="2" t="s">
         <v>35</v>
       </c>
     </row>
@@ -5590,7 +5617,7 @@
       <c r="B219" t="s">
         <v>367</v>
       </c>
-      <c r="C219" s="4" t="s">
+      <c r="C219" s="3" t="s">
         <v>419</v>
       </c>
     </row>
@@ -5601,7 +5628,7 @@
       <c r="B220" t="s">
         <v>368</v>
       </c>
-      <c r="C220" s="3" t="s">
+      <c r="C220" s="2" t="s">
         <v>420</v>
       </c>
     </row>
@@ -5612,7 +5639,7 @@
       <c r="B221" t="s">
         <v>369</v>
       </c>
-      <c r="C221" s="4" t="s">
+      <c r="C221" s="3" t="s">
         <v>421</v>
       </c>
       <c r="E221" t="s">
@@ -5629,7 +5656,7 @@
       <c r="B222" t="s">
         <v>370</v>
       </c>
-      <c r="C222" s="4" t="s">
+      <c r="C222" s="3" t="s">
         <v>422</v>
       </c>
       <c r="F222" t="s">
@@ -5646,7 +5673,7 @@
       <c r="B223" t="s">
         <v>371</v>
       </c>
-      <c r="C223" s="4" t="s">
+      <c r="C223" s="3" t="s">
         <v>423</v>
       </c>
     </row>
@@ -5657,43 +5684,43 @@
       <c r="B224" t="s">
         <v>372</v>
       </c>
-      <c r="C224" s="4" t="s">
+      <c r="C224" s="3" t="s">
         <v>424</v>
       </c>
       <c r="F224" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="225" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="225" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A225" t="s">
         <v>326</v>
       </c>
       <c r="B225" t="s">
         <v>373</v>
       </c>
-      <c r="C225" s="3" t="s">
+      <c r="C225" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="226" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="226" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A226" t="s">
         <v>326</v>
       </c>
       <c r="B226" t="s">
         <v>374</v>
       </c>
-      <c r="C226" s="4" t="s">
+      <c r="C226" s="3" t="s">
         <v>425</v>
       </c>
     </row>
-    <row r="227" spans="1:6" ht="34" x14ac:dyDescent="0.2">
+    <row r="227" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A227" t="s">
         <v>326</v>
       </c>
       <c r="B227" t="s">
         <v>375</v>
       </c>
-      <c r="C227" s="4" t="s">
+      <c r="C227" s="3" t="s">
         <v>426</v>
       </c>
       <c r="E227" t="s">
@@ -5703,355 +5730,364 @@
         <v>14</v>
       </c>
     </row>
-    <row r="228" spans="1:6" ht="34" x14ac:dyDescent="0.2">
+    <row r="228" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A228" t="s">
         <v>326</v>
       </c>
       <c r="B228" t="s">
         <v>376</v>
       </c>
-      <c r="C228" s="4" t="s">
+      <c r="C228" s="3" t="s">
         <v>427</v>
       </c>
       <c r="E228" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="229" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="229" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A229" t="s">
         <v>326</v>
       </c>
       <c r="B229" t="s">
         <v>377</v>
       </c>
-      <c r="C229" s="4" t="s">
+      <c r="C229" s="3" t="s">
         <v>428</v>
       </c>
       <c r="F229" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="230" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+    <row r="230" spans="1:12" ht="51" x14ac:dyDescent="0.2">
       <c r="A230" t="s">
         <v>326</v>
       </c>
       <c r="B230" t="s">
         <v>378</v>
       </c>
-      <c r="C230" s="4" t="s">
+      <c r="C230" s="3" t="s">
         <v>429</v>
       </c>
       <c r="D230" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="231" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="231" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A231" t="s">
         <v>326</v>
       </c>
       <c r="B231" t="s">
         <v>379</v>
       </c>
-      <c r="C231" s="4" t="s">
+      <c r="C231" s="3" t="s">
         <v>430</v>
       </c>
       <c r="F231" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="232" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="232" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A232" t="s">
         <v>326</v>
       </c>
       <c r="B232" t="s">
         <v>380</v>
       </c>
-      <c r="C232" s="3" t="s">
+      <c r="C232" s="2" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="233" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="233" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A233" t="s">
         <v>326</v>
       </c>
       <c r="B233" t="s">
         <v>381</v>
       </c>
-      <c r="C233" s="3" t="s">
+      <c r="C233" s="2" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="234" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="234" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A234" t="s">
         <v>326</v>
       </c>
       <c r="B234" t="s">
         <v>382</v>
       </c>
-      <c r="C234" s="4" t="s">
+      <c r="C234" s="3" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="235" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="235" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A235" t="s">
         <v>326</v>
       </c>
       <c r="B235" t="s">
         <v>383</v>
       </c>
-      <c r="C235" s="4" t="s">
+      <c r="C235" s="3" t="s">
         <v>431</v>
       </c>
       <c r="F235" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="236" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="236" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A236" t="s">
         <v>326</v>
       </c>
       <c r="B236" t="s">
         <v>384</v>
       </c>
-      <c r="C236" s="4" t="s">
+      <c r="C236" s="3" t="s">
         <v>432</v>
       </c>
       <c r="F236" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="237" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+      <c r="L236" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="237" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A237" t="s">
         <v>326</v>
       </c>
       <c r="B237" t="s">
         <v>385</v>
       </c>
-      <c r="C237" s="4" t="s">
+      <c r="C237" s="3" t="s">
         <v>433</v>
       </c>
       <c r="F237" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="238" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+      <c r="L237" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="238" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A238" t="s">
         <v>326</v>
       </c>
       <c r="B238" t="s">
         <v>386</v>
       </c>
-      <c r="C238" s="3" t="s">
+      <c r="C238" s="2" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="239" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="239" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A239" t="s">
         <v>326</v>
       </c>
       <c r="B239" t="s">
         <v>387</v>
       </c>
-      <c r="C239" s="4" t="s">
+      <c r="C239" s="3" t="s">
         <v>434</v>
       </c>
     </row>
-    <row r="240" spans="1:6" ht="34" x14ac:dyDescent="0.2">
+    <row r="240" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A240" t="s">
         <v>326</v>
       </c>
       <c r="B240" t="s">
         <v>388</v>
       </c>
-      <c r="C240" s="4" t="s">
+      <c r="C240" s="3" t="s">
         <v>435</v>
       </c>
       <c r="D240" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="241" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="241" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A241" t="s">
         <v>326</v>
       </c>
       <c r="B241" t="s">
         <v>389</v>
       </c>
-      <c r="C241" s="4" t="s">
+      <c r="C241" s="3" t="s">
         <v>436</v>
       </c>
-    </row>
-    <row r="242" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="L241" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="242" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A242" t="s">
         <v>326</v>
       </c>
       <c r="B242" t="s">
         <v>390</v>
       </c>
-      <c r="C242" s="3" t="s">
+      <c r="C242" s="2" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="243" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+    <row r="243" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A243" t="s">
         <v>437</v>
       </c>
       <c r="B243" t="s">
         <v>438</v>
       </c>
-      <c r="C243" s="4" t="s">
+      <c r="C243" s="3" t="s">
         <v>502</v>
       </c>
       <c r="E243" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="244" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="244" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A244" t="s">
         <v>437</v>
       </c>
       <c r="B244" t="s">
         <v>439</v>
       </c>
-      <c r="C244" s="3" t="s">
+      <c r="C244" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="245" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="245" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A245" t="s">
         <v>437</v>
       </c>
       <c r="B245" t="s">
         <v>440</v>
       </c>
-      <c r="C245" s="4" t="s">
+      <c r="C245" s="3" t="s">
         <v>503</v>
       </c>
       <c r="E245" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="246" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="246" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A246" t="s">
         <v>437</v>
       </c>
       <c r="B246" t="s">
         <v>441</v>
       </c>
-      <c r="C246" s="4" t="s">
+      <c r="C246" s="3" t="s">
         <v>504</v>
       </c>
     </row>
-    <row r="247" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="247" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A247" t="s">
         <v>437</v>
       </c>
       <c r="B247" t="s">
         <v>442</v>
       </c>
-      <c r="C247" s="3" t="s">
+      <c r="C247" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="248" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+    <row r="248" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A248" t="s">
         <v>437</v>
       </c>
       <c r="B248" t="s">
         <v>443</v>
       </c>
-      <c r="C248" s="4" t="s">
+      <c r="C248" s="3" t="s">
         <v>505</v>
       </c>
       <c r="E248" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="249" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="249" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A249" t="s">
         <v>437</v>
       </c>
       <c r="B249" t="s">
         <v>444</v>
       </c>
-      <c r="C249" s="3" t="s">
+      <c r="C249" s="2" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="250" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+    <row r="250" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A250" t="s">
         <v>437</v>
       </c>
       <c r="B250" t="s">
         <v>445</v>
       </c>
-      <c r="C250" s="4" t="s">
+      <c r="C250" s="3" t="s">
         <v>506</v>
       </c>
     </row>
-    <row r="251" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="251" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A251" t="s">
         <v>437</v>
       </c>
       <c r="B251" t="s">
         <v>446</v>
       </c>
-      <c r="C251" s="3" t="s">
+      <c r="C251" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="252" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="252" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A252" t="s">
         <v>437</v>
       </c>
       <c r="B252" t="s">
         <v>447</v>
       </c>
-      <c r="C252" s="4" t="s">
+      <c r="C252" s="3" t="s">
         <v>507</v>
       </c>
     </row>
-    <row r="253" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="253" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A253" t="s">
         <v>437</v>
       </c>
       <c r="B253" t="s">
         <v>448</v>
       </c>
-      <c r="C253" s="3" t="s">
+      <c r="C253" s="2" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="254" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="254" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A254" t="s">
         <v>437</v>
       </c>
       <c r="B254" t="s">
         <v>449</v>
       </c>
-      <c r="C254" s="3" t="s">
+      <c r="C254" s="2" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="255" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="255" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A255" t="s">
         <v>437</v>
       </c>
       <c r="B255" t="s">
         <v>450</v>
       </c>
-      <c r="C255" s="3" t="s">
+      <c r="C255" s="2" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="256" spans="1:5" ht="85" x14ac:dyDescent="0.2">
+    <row r="256" spans="1:12" ht="85" x14ac:dyDescent="0.2">
       <c r="A256" t="s">
         <v>437</v>
       </c>
       <c r="B256" t="s">
         <v>451</v>
       </c>
-      <c r="C256" s="4" t="s">
+      <c r="C256" s="3" t="s">
         <v>508</v>
       </c>
     </row>
@@ -6062,7 +6098,7 @@
       <c r="B257" t="s">
         <v>452</v>
       </c>
-      <c r="C257" s="3" t="s">
+      <c r="C257" s="2" t="s">
         <v>400</v>
       </c>
     </row>
@@ -6073,7 +6109,7 @@
       <c r="B258" t="s">
         <v>453</v>
       </c>
-      <c r="C258" s="3"/>
+      <c r="C258" s="2"/>
     </row>
     <row r="259" spans="1:6" ht="34" x14ac:dyDescent="0.2">
       <c r="A259" t="s">
@@ -6082,7 +6118,7 @@
       <c r="B259" t="s">
         <v>454</v>
       </c>
-      <c r="C259" s="4" t="s">
+      <c r="C259" s="3" t="s">
         <v>509</v>
       </c>
       <c r="E259" t="s">
@@ -6096,7 +6132,7 @@
       <c r="B260" t="s">
         <v>455</v>
       </c>
-      <c r="C260" s="4" t="s">
+      <c r="C260" s="3" t="s">
         <v>510</v>
       </c>
     </row>
@@ -6107,7 +6143,7 @@
       <c r="B261" t="s">
         <v>456</v>
       </c>
-      <c r="C261" s="4" t="s">
+      <c r="C261" s="3" t="s">
         <v>511</v>
       </c>
       <c r="E261" t="s">
@@ -6121,7 +6157,7 @@
       <c r="B262" t="s">
         <v>457</v>
       </c>
-      <c r="C262" s="3" t="s">
+      <c r="C262" s="2" t="s">
         <v>29</v>
       </c>
     </row>
@@ -6132,7 +6168,7 @@
       <c r="B263" t="s">
         <v>458</v>
       </c>
-      <c r="C263" s="3" t="s">
+      <c r="C263" s="2" t="s">
         <v>400</v>
       </c>
     </row>
@@ -6143,7 +6179,7 @@
       <c r="B264" t="s">
         <v>459</v>
       </c>
-      <c r="C264" s="4" t="s">
+      <c r="C264" s="3" t="s">
         <v>512</v>
       </c>
     </row>
@@ -6154,7 +6190,7 @@
       <c r="B265" t="s">
         <v>460</v>
       </c>
-      <c r="C265" s="3" t="s">
+      <c r="C265" s="2" t="s">
         <v>64</v>
       </c>
     </row>
@@ -6165,7 +6201,7 @@
       <c r="B266" t="s">
         <v>461</v>
       </c>
-      <c r="C266" s="4" t="s">
+      <c r="C266" s="3" t="s">
         <v>513</v>
       </c>
       <c r="F266" t="s">
@@ -6179,7 +6215,7 @@
       <c r="B267" t="s">
         <v>462</v>
       </c>
-      <c r="C267" s="3" t="s">
+      <c r="C267" s="2" t="s">
         <v>35</v>
       </c>
     </row>
@@ -6190,7 +6226,7 @@
       <c r="B268" t="s">
         <v>463</v>
       </c>
-      <c r="C268" s="4" t="s">
+      <c r="C268" s="3" t="s">
         <v>514</v>
       </c>
       <c r="E268" t="s">
@@ -6204,7 +6240,7 @@
       <c r="B269" t="s">
         <v>464</v>
       </c>
-      <c r="C269" s="3" t="s">
+      <c r="C269" s="2" t="s">
         <v>400</v>
       </c>
     </row>
@@ -6215,7 +6251,7 @@
       <c r="B270" t="s">
         <v>465</v>
       </c>
-      <c r="C270" s="3" t="s">
+      <c r="C270" s="2" t="s">
         <v>29</v>
       </c>
     </row>
@@ -6226,7 +6262,7 @@
       <c r="B271" t="s">
         <v>466</v>
       </c>
-      <c r="C271" s="3" t="s">
+      <c r="C271" s="2" t="s">
         <v>400</v>
       </c>
     </row>
@@ -6237,387 +6273,420 @@
       <c r="B272" t="s">
         <v>467</v>
       </c>
-      <c r="C272" s="4" t="s">
+      <c r="C272" s="3" t="s">
         <v>515</v>
       </c>
     </row>
-    <row r="273" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="273" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A273" t="s">
         <v>437</v>
       </c>
       <c r="B273" t="s">
         <v>468</v>
       </c>
-      <c r="C273" s="4" t="s">
+      <c r="C273" s="3" t="s">
         <v>516</v>
       </c>
       <c r="F273" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="274" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+      <c r="L273" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="274" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A274" t="s">
         <v>437</v>
       </c>
       <c r="B274" t="s">
         <v>469</v>
       </c>
-      <c r="C274" s="4" t="s">
+      <c r="C274" s="3" t="s">
         <v>517</v>
       </c>
       <c r="F274" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="275" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+      <c r="L274" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="275" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A275" t="s">
         <v>437</v>
       </c>
       <c r="B275" t="s">
         <v>470</v>
       </c>
-      <c r="C275" s="4" t="s">
+      <c r="C275" s="3" t="s">
         <v>518</v>
       </c>
       <c r="F275" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="276" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="276" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A276" t="s">
         <v>437</v>
       </c>
       <c r="B276" t="s">
         <v>471</v>
       </c>
-      <c r="C276" s="4" t="s">
+      <c r="C276" s="3" t="s">
         <v>519</v>
       </c>
-    </row>
-    <row r="277" spans="1:6" ht="68" x14ac:dyDescent="0.2">
+      <c r="M276" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="277" spans="1:13" ht="68" x14ac:dyDescent="0.2">
       <c r="A277" t="s">
         <v>437</v>
       </c>
       <c r="B277" t="s">
         <v>472</v>
       </c>
-      <c r="C277" s="4" t="s">
+      <c r="C277" s="3" t="s">
         <v>520</v>
       </c>
       <c r="F277" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="278" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="278" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A278" t="s">
         <v>437</v>
       </c>
       <c r="B278" t="s">
         <v>473</v>
       </c>
-      <c r="C278" s="3" t="s">
+      <c r="C278" s="2" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="279" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="279" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A279" t="s">
         <v>437</v>
       </c>
       <c r="B279" t="s">
         <v>474</v>
       </c>
-      <c r="C279" s="4" t="s">
+      <c r="C279" s="3" t="s">
         <v>521</v>
       </c>
       <c r="F279" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="280" spans="1:6" ht="34" x14ac:dyDescent="0.2">
+      <c r="L279" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="280" spans="1:13" ht="34" x14ac:dyDescent="0.2">
       <c r="A280" t="s">
         <v>437</v>
       </c>
       <c r="B280" t="s">
         <v>475</v>
       </c>
-      <c r="C280" s="4" t="s">
+      <c r="C280" s="3" t="s">
         <v>522</v>
       </c>
     </row>
-    <row r="281" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="281" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A281" t="s">
         <v>437</v>
       </c>
       <c r="B281" t="s">
         <v>476</v>
       </c>
-      <c r="C281" s="3" t="s">
+      <c r="C281" s="2" t="s">
         <v>523</v>
       </c>
     </row>
-    <row r="282" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="282" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A282" t="s">
         <v>437</v>
       </c>
       <c r="B282" t="s">
         <v>477</v>
       </c>
-      <c r="C282" s="3" t="s">
+      <c r="C282" s="2" t="s">
         <v>524</v>
       </c>
     </row>
-    <row r="283" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="283" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A283" t="s">
         <v>437</v>
       </c>
       <c r="B283" t="s">
         <v>478</v>
       </c>
-      <c r="C283" s="3" t="s">
+      <c r="C283" s="2" t="s">
         <v>523</v>
       </c>
     </row>
-    <row r="284" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="284" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A284" t="s">
         <v>437</v>
       </c>
       <c r="B284" t="s">
         <v>479</v>
       </c>
-      <c r="C284" s="3" t="s">
+      <c r="C284" s="2" t="s">
         <v>523</v>
       </c>
     </row>
-    <row r="285" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="285" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A285" t="s">
         <v>437</v>
       </c>
       <c r="B285" t="s">
         <v>480</v>
       </c>
-      <c r="C285" s="3" t="s">
+      <c r="C285" s="2" t="s">
         <v>523</v>
       </c>
     </row>
-    <row r="286" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="286" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A286" t="s">
         <v>437</v>
       </c>
       <c r="B286" t="s">
         <v>481</v>
       </c>
-      <c r="C286" s="3" t="s">
+      <c r="C286" s="2" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="287" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="287" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A287" t="s">
         <v>437</v>
       </c>
       <c r="B287" t="s">
         <v>482</v>
       </c>
-      <c r="C287" s="3" t="s">
+      <c r="C287" s="2" t="s">
         <v>525</v>
       </c>
     </row>
-    <row r="288" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="288" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A288" t="s">
         <v>437</v>
       </c>
       <c r="B288" t="s">
         <v>491</v>
       </c>
-      <c r="C288" s="3" t="s">
+      <c r="C288" s="2" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="289" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="289" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A289" t="s">
         <v>437</v>
       </c>
       <c r="B289" t="s">
         <v>483</v>
       </c>
-      <c r="C289" s="4" t="s">
+      <c r="C289" s="3" t="s">
         <v>517</v>
       </c>
       <c r="F289" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="290" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+      <c r="L289" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="290" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A290" t="s">
         <v>437</v>
       </c>
       <c r="B290" t="s">
         <v>484</v>
       </c>
-      <c r="C290" s="4" t="s">
+      <c r="C290" s="3" t="s">
         <v>295</v>
       </c>
     </row>
-    <row r="291" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="291" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A291" t="s">
         <v>437</v>
       </c>
       <c r="B291" t="s">
         <v>485</v>
       </c>
-      <c r="C291" s="4" t="s">
+      <c r="C291" s="3" t="s">
         <v>526</v>
       </c>
       <c r="F291" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="292" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+      <c r="L291" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="292" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A292" t="s">
         <v>437</v>
       </c>
       <c r="B292" t="s">
         <v>486</v>
       </c>
-      <c r="C292" s="4" t="s">
+      <c r="C292" s="3" t="s">
         <v>527</v>
       </c>
       <c r="F292" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="293" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+      <c r="L292" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="293" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A293" t="s">
         <v>437</v>
       </c>
       <c r="B293" t="s">
         <v>487</v>
       </c>
-      <c r="C293" s="4" t="s">
+      <c r="C293" s="3" t="s">
         <v>528</v>
       </c>
-    </row>
-    <row r="294" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+      <c r="M293" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="294" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A294" t="s">
         <v>437</v>
       </c>
       <c r="B294" t="s">
         <v>488</v>
       </c>
-      <c r="C294" s="4" t="s">
+      <c r="C294" s="3" t="s">
         <v>295</v>
       </c>
     </row>
-    <row r="295" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="295" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A295" t="s">
         <v>437</v>
       </c>
       <c r="B295" t="s">
         <v>489</v>
       </c>
-      <c r="C295" s="4" t="s">
+      <c r="C295" s="3" t="s">
         <v>529</v>
       </c>
-    </row>
-    <row r="296" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+      <c r="M295" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="296" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A296" t="s">
         <v>437</v>
       </c>
       <c r="B296" t="s">
         <v>490</v>
       </c>
-      <c r="C296" s="3" t="s">
+      <c r="C296" s="2" t="s">
         <v>523</v>
       </c>
     </row>
-    <row r="297" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="297" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A297" t="s">
         <v>437</v>
       </c>
       <c r="B297" t="s">
         <v>492</v>
       </c>
-      <c r="C297" s="3" t="s">
+      <c r="C297" s="2" t="s">
         <v>523</v>
       </c>
     </row>
-    <row r="298" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="298" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A298" t="s">
         <v>437</v>
       </c>
       <c r="B298" t="s">
         <v>493</v>
       </c>
-      <c r="C298" s="4" t="s">
+      <c r="C298" s="3" t="s">
         <v>411</v>
       </c>
     </row>
-    <row r="299" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="299" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A299" t="s">
         <v>437</v>
       </c>
       <c r="B299" t="s">
         <v>494</v>
       </c>
-      <c r="C299" s="4" t="s">
+      <c r="C299" s="3" t="s">
         <v>530</v>
       </c>
       <c r="F299" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="300" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+      <c r="L299" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="300" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A300" t="s">
         <v>437</v>
       </c>
       <c r="B300" t="s">
         <v>495</v>
       </c>
-      <c r="C300" s="3" t="s">
+      <c r="C300" s="2" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="301" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="301" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A301" t="s">
         <v>437</v>
       </c>
       <c r="B301" t="s">
         <v>496</v>
       </c>
-      <c r="C301" s="3" t="s">
+      <c r="C301" s="2" t="s">
         <v>531</v>
       </c>
     </row>
-    <row r="302" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="302" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A302" t="s">
         <v>437</v>
       </c>
       <c r="B302" t="s">
         <v>497</v>
       </c>
-      <c r="C302" s="3" t="s">
+      <c r="C302" s="2" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="303" spans="1:6" ht="34" x14ac:dyDescent="0.2">
+    <row r="303" spans="1:13" ht="34" x14ac:dyDescent="0.2">
       <c r="A303" t="s">
         <v>437</v>
       </c>
       <c r="B303" t="s">
         <v>498</v>
       </c>
-      <c r="C303" s="4" t="s">
+      <c r="C303" s="3" t="s">
         <v>532</v>
       </c>
     </row>
-    <row r="304" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="304" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A304" t="s">
         <v>437</v>
       </c>
       <c r="B304" t="s">
         <v>499</v>
       </c>
-      <c r="C304" s="4" t="s">
+      <c r="C304" s="3" t="s">
         <v>533</v>
+      </c>
+      <c r="M304" t="s">
+        <v>539</v>
       </c>
     </row>
     <row r="305" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -6627,7 +6696,7 @@
       <c r="B305" t="s">
         <v>500</v>
       </c>
-      <c r="C305" s="4" t="s">
+      <c r="C305" s="3" t="s">
         <v>534</v>
       </c>
       <c r="E305" t="s">
@@ -6641,7 +6710,7 @@
       <c r="B306" t="s">
         <v>501</v>
       </c>
-      <c r="C306" s="4" t="s">
+      <c r="C306" s="3" t="s">
         <v>535</v>
       </c>
     </row>

</xml_diff>